<commit_message>
feat: CRUD de Autoridades e estabilização do app Desktop
</commit_message>
<xml_diff>
--- a/almoxarifado/terminal_balcao/planilhas_consolidadas/Almoxarifado_ARGUS_Consolidado.xlsx
+++ b/almoxarifado/terminal_balcao/planilhas_consolidadas/Almoxarifado_ARGUS_Consolidado.xlsx
@@ -749,13 +749,13 @@
         <v>100</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>100</v>
+        <v>285</v>
       </c>
       <c r="I7" s="8" t="n">
         <v>25</v>
@@ -1880,10 +1880,10 @@
         <v>0</v>
       </c>
       <c r="G31" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H31" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I31" s="8" t="n">
         <v>2</v>
@@ -2864,10 +2864,10 @@
         <v>1</v>
       </c>
       <c r="F52" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G52" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H52" s="5" t="n">
         <v>1</v>
@@ -4321,13 +4321,13 @@
         <v>180</v>
       </c>
       <c r="F83" s="8" t="n">
-        <v>0</v>
+        <v>11.25</v>
       </c>
       <c r="G83" s="8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H83" s="8" t="n">
-        <v>180</v>
+        <v>187.25</v>
       </c>
       <c r="I83" s="8" t="n">
         <v>3.75</v>
@@ -4827,7 +4827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4914,6 +4914,162 @@
         </is>
       </c>
     </row>
+    <row r="4" ht="19" customHeight="1">
+      <c r="A4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>14/09/2026 18:16</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>RETORNO</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>DEVOLUÇÃO: GABRIEL COLARES</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>MARRETA 1,00KG</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>UN</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>UN</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>POLO GERAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="19" customHeight="1">
+      <c r="A5" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>14/09/2026 18:16</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>RETORNO-SOBRA</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>DEVOLUÇÃO: COLABORADORA ALMOXARIFADO</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>TINTA ACRILICA STANDART BRANCO NEVE 15L</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>FRAÇÃO</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="7" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO PREDIAL / POLO GERAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="19" customHeight="1">
+      <c r="A6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>NF-TESTE-01</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>DISTRIBUIDORA ELETRICA</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>CABO FLEXIVEL 1X 1,5 VERDE  100MT</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>ROLO 100M</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="n">
+        <v>180</v>
+      </c>
+      <c r="K6" s="5" t="n">
+        <v>360</v>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO PREDIAL / POLO GERAL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:K1"/>
@@ -4928,7 +5084,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5003,6 +5159,206 @@
         </is>
       </c>
     </row>
+    <row r="4" ht="19" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>SAI-EMP-2026-0002</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>15/09/2026 19:05</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>DESEMPENADEIRA DE AÇO LISA</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>UN</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>GABRIEL ALMEIDA SANTOS DE OLIVEIRA</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>CV 007/2022 AX ACADEMY</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>EMPRÉSTIMO DE FERRAMENTA</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>EMPRESTIMO_FERRAMENTA</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>TERMO-2026/0002</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="19" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>SAI-EMP-2026-0001</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>14/09/2026 18:16</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>MARRETA 1,00KG</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>UN</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>GABRIEL COLARES</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>P&amp;D INDÚSTRIA 4.0</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>EMPRÉSTIMO DE FERRAMENTA</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>EMPRESTIMO_FERRAMENTA</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>TERMO-2026/0001</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="19" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>SAI-2026-0002</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>14/09/2026 18:16</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>TINTA ACRILICA STANDART BRANCO NEVE 15L</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>COLABORADORA ALMOXARIFADO</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO PREDIAL / POLO GERAL</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>SALA DE SERVIDORES</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>CONSUMO</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>REC-2026/0002</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="19" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>SAI-2026-0001</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>14/09/2026 18:16</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>CABO FLEXIVEL 1X 1,5 VERDE  100MT</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>GABRIEL COLARES</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO PREDIAL / POLO GERAL</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>LSCN - LABORATÓRIO</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>CONSUMO</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>REC-2026/0001</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
@@ -5017,7 +5373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5086,6 +5442,88 @@
         </is>
       </c>
     </row>
+    <row r="4" ht="19" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>EMP-2026/0002</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>DESEMPENADEIRA DE AÇO LISA</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>GABRIEL ALMEIDA SANTOS DE OLIVEIRA</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>CV 007/2022 AX ACADEMY</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>15/09/2026</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>2027-01-11</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>EM USO</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr"/>
+      <c r="I4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5" ht="19" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>EMP-2026/0001</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>MARRETA 1,00KG</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>GABRIEL COLARES</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>P&amp;D INDÚSTRIA 4.0</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr"/>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>DEVOLVIDO</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>14/09/2026 18:16</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>Devolvido em perfeito estado</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
@@ -5100,12 +5538,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:D65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -5118,15 +5557,20 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>SOLICITANTES</t>
+          <t>SOLICITANTE (NOME)</t>
         </is>
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
+          <t>SOLICITANTE (CPF)</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
           <t>PROJETOS</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="D3" s="10" t="inlineStr">
         <is>
           <t>AMBIENTES</t>
         </is>
@@ -5135,15 +5579,20 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>ALISON SILVA DA CUNHA CPF:704.131.172-43</t>
+          <t>ALISON SILVA DA CUNHA</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>BIO CAROÇO (EDITAL FAEPI 072/2026)</t>
+          <t>70413117243</t>
         </is>
       </c>
       <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>BIO CAROÇO</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
         <is>
           <t>ALMOXARIFADO CENTRAL</t>
         </is>
@@ -5155,12 +5604,13 @@
           <t>ANDRÉ BELTRÃO DE LUCENA</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr"/>
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>CANTEIROHUB</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="D5" s="11" t="inlineStr">
         <is>
           <t>ALMOXARIFADO MANUTENÇÃO</t>
         </is>
@@ -5172,12 +5622,13 @@
           <t>ANTÔNIO FERREIRA DOS SANTOS JUNIOR</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr"/>
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>CV 001/2020 SAGEMCON</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="D6" s="11" t="inlineStr">
         <is>
           <t>COPA</t>
         </is>
@@ -5186,15 +5637,20 @@
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
         <is>
-          <t>BRENDA LIMA CEZAR CPF:702.298.512-07</t>
+          <t>BRENDA LIMA CEZAR</t>
         </is>
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
+          <t>70229851207</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
           <t>CV 001/2022 IOT</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="D7" s="11" t="inlineStr">
         <is>
           <t>CORREDORES</t>
         </is>
@@ -5206,12 +5662,13 @@
           <t>CARLOS GOMES VASCONCELOS</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr"/>
+      <c r="C8" s="11" t="inlineStr">
         <is>
           <t>CV 002/2023 ERGO SALUS</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="D8" s="11" t="inlineStr">
         <is>
           <t>ESPAÇO MAKER</t>
         </is>
@@ -5223,12 +5680,13 @@
           <t>COLABORADORA ALMOXARIFADO</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr"/>
+      <c r="C9" s="11" t="inlineStr">
         <is>
           <t>CV 007/2022 AX ACADEMY</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="D9" s="11" t="inlineStr">
         <is>
           <t>LABORATÓRIO LABCODING</t>
         </is>
@@ -5237,15 +5695,20 @@
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>DIEGO CAMARA SALES  CPF: 880.620.822-53</t>
+          <t>DIEGO CAMARA SALES</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
+          <t>88062082253</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
           <t>CV 008/2021 FOGO BIO</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="D10" s="11" t="inlineStr">
         <is>
           <t>LABORATÓRIO LEMAS</t>
         </is>
@@ -5257,12 +5720,13 @@
           <t>EDUARDO PALHARES JUNIOR</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr"/>
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>CV 011/2021 TELECOM</t>
         </is>
       </c>
-      <c r="C11" s="11" t="inlineStr">
+      <c r="D11" s="11" t="inlineStr">
         <is>
           <t>LABORATÓRIO LPH</t>
         </is>
@@ -5274,12 +5738,13 @@
           <t>ELIENAI NOGUEIRA</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr"/>
+      <c r="C12" s="11" t="inlineStr">
         <is>
           <t>CV 016/2022 COELMATIC</t>
         </is>
       </c>
-      <c r="C12" s="11" t="inlineStr">
+      <c r="D12" s="11" t="inlineStr">
         <is>
           <t>LABORATÓRIO LRI</t>
         </is>
@@ -5291,12 +5756,13 @@
           <t>EQUIPE DE MANUTENÇÃO</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr"/>
+      <c r="C13" s="11" t="inlineStr">
         <is>
           <t>MANUTENÇÃO PREDIAL / POLO GERAL</t>
         </is>
       </c>
-      <c r="C13" s="11" t="inlineStr">
+      <c r="D13" s="11" t="inlineStr">
         <is>
           <t>LABORATÓRIO LSCN</t>
         </is>
@@ -5308,12 +5774,13 @@
           <t>EQUIPE P&amp;D</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr"/>
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>P&amp;D INDÚSTRIA 4.0</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
+      <c r="D14" s="11" t="inlineStr">
         <is>
           <t>LSCN - LABORATÓRIO</t>
         </is>
@@ -5322,15 +5789,20 @@
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>ERONICE VIEIRA DE MOURA - CPF: 961.946.932-15</t>
+          <t>ERONICE VIEIRA DE MOURA</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
+          <t>96194693215</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
           <t>PIBIC / INICIAÇÃO CIENTÍFICA</t>
         </is>
       </c>
-      <c r="C15" s="11" t="inlineStr">
+      <c r="D15" s="11" t="inlineStr">
         <is>
           <t>OFICINA MECÂNICA</t>
         </is>
@@ -5339,10 +5811,15 @@
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>FRANCISCO CORDEIRO DA SILVA FELIX CPF:019.222.342-90</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="inlineStr">
+          <t>FRANCISCO CORDEIRO DA SILVA FELIX</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>01922234290</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
         <is>
           <t>RECEPÇÃO</t>
         </is>
@@ -5351,10 +5828,15 @@
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>FRANCISCO XAVIER NOBRE CPF:050.406.403-74</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="inlineStr">
+          <t>FRANCISCO XAVIER NOBRE</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>05040640374</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
         <is>
           <t>SALA DA ADMINISTRAÇÃO</t>
         </is>
@@ -5363,10 +5845,15 @@
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>GABRIEL ALMEIDA SANTOS DE OLIVEIRA. CPF:985.540.262- 68</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="inlineStr">
+          <t>GABRIEL ALMEIDA SANTOS DE OLIVEIRA</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>98554026268</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
         <is>
           <t>SALA DA CPO</t>
         </is>
@@ -5378,7 +5865,8 @@
           <t>GABRIEL COLARES</t>
         </is>
       </c>
-      <c r="C19" s="11" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr"/>
+      <c r="D19" s="11" t="inlineStr">
         <is>
           <t>SALA DA DIRETORIA</t>
         </is>
@@ -5390,7 +5878,8 @@
           <t>GABRIEL DE SOUZA LEITÃO</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
+      <c r="B20" s="11" t="inlineStr"/>
+      <c r="D20" s="11" t="inlineStr">
         <is>
           <t>SALA DA PROSPECÇÃO</t>
         </is>
@@ -5399,10 +5888,15 @@
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>GEZIEL  SENA  COLARES,  CPF:  834.038.762-68</t>
-        </is>
-      </c>
-      <c r="C21" s="11" t="inlineStr">
+          <t>GEZIEL  SENA  COLARES</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>83403876268</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
         <is>
           <t>SALA DE REUNIÃO</t>
         </is>
@@ -5414,7 +5908,8 @@
           <t>GEZIEL SENA COLARES</t>
         </is>
       </c>
-      <c r="C22" s="11" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr"/>
+      <c r="D22" s="11" t="inlineStr">
         <is>
           <t>SALA DE SERVIDORES</t>
         </is>
@@ -5423,10 +5918,15 @@
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
         <is>
-          <t>GILBERT BREVES MARTINS CPF: 337.836.672-91</t>
-        </is>
-      </c>
-      <c r="C23" s="11" t="inlineStr">
+          <t>GILBERT BREVES MARTINS</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>33783667291</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
         <is>
           <t>SALA DO TI</t>
         </is>
@@ -5438,7 +5938,8 @@
           <t>GÉRLISON SAMPAIO DA SILVA</t>
         </is>
       </c>
-      <c r="C24" s="11" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr"/>
+      <c r="D24" s="11" t="inlineStr">
         <is>
           <t>SUBESTAÇÃO ELÉTRICA</t>
         </is>
@@ -5450,7 +5951,8 @@
           <t>HILLERMANN FERREIRA OSMÍDIO LIMA</t>
         </is>
       </c>
-      <c r="C25" s="11" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr"/>
+      <c r="D25" s="11" t="inlineStr">
         <is>
           <t>ÁREA EXTERNA</t>
         </is>
@@ -5459,9 +5961,10 @@
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>HILLERMANN FERREIRA OSMÍDIO LIMA  SIAPE:1506333</t>
-        </is>
-      </c>
+          <t>HILLERMANN FERREIRA OSMÍDIO LIMA</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
@@ -5469,11 +5972,17 @@
           <t>JAIDSON BRANDÃO DA COSTA, DIR. IFAM  MANACAPURU (SOLITAR)</t>
         </is>
       </c>
+      <c r="B27" s="11" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>JOSÉ JOSIMAR SOARES CPF: 884.376.254-72</t>
+          <t>JOSÉ JOSIMAR SOARES</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>88437625472</t>
         </is>
       </c>
     </row>
@@ -5483,11 +5992,17 @@
           <t>JOSÉ PINHEIRO DE QUEIROZ NETO</t>
         </is>
       </c>
+      <c r="B29" s="11" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>JULIANA BRITO FEITOSA CPF:021.614.462-07</t>
+          <t>JULIANA BRITO FEITOSA</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>02161446207</t>
         </is>
       </c>
     </row>
@@ -5497,11 +6012,17 @@
           <t>JULIANE DE OLIVEIRA SILVA</t>
         </is>
       </c>
+      <c r="B31" s="11" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>KETHELEN PALMA MONTEIRO CPF: 016.997.852-44</t>
+          <t>KETHELEN PALMA MONTEIRO</t>
+        </is>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>01699785244</t>
         </is>
       </c>
     </row>
@@ -5511,39 +6032,61 @@
           <t>LABORATORIO DE HARDWARE</t>
         </is>
       </c>
+      <c r="B33" s="11" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>LANIER MENEZES DOS SANTOS CPF: 948.621.502-25</t>
+          <t>LANIER MENEZES DOS SANTOS</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>94862150225</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="inlineStr">
         <is>
-          <t>LANIER MENEZES DOS SANTOS CPF: 948.621.502-26</t>
+          <t>LANIER MENEZES DOS SANTOS</t>
+        </is>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>94862150226</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>LAURA MICHAELLA BATISTA RIBEIRO</t>
+          <t>LAURA MICHAELLA</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>88303667220</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="11" t="inlineStr">
         <is>
-          <t>LAURA MICHAELLA CPF/ 883.036.672-20</t>
-        </is>
-      </c>
+          <t>LAURA MICHAELLA BATISTA RIBEIRO</t>
+        </is>
+      </c>
+      <c r="B37" s="11" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="11" t="inlineStr">
         <is>
-          <t>LAWANY DA SILVA SOUZA, CPF 048.407.532-29</t>
+          <t>LAWANY DA SILVA SOUZA</t>
+        </is>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>04840753229</t>
         </is>
       </c>
     </row>
@@ -5553,11 +6096,17 @@
           <t>LUANNE OLIVEIRA LEITE</t>
         </is>
       </c>
+      <c r="B39" s="11" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="11" t="inlineStr">
         <is>
-          <t>LUCAS RODRIGUES DE SOUSA CPF: 048.484.832-12</t>
+          <t>LUCAS RODRIGUES DE SOUSA</t>
+        </is>
+      </c>
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>04848483212</t>
         </is>
       </c>
     </row>
@@ -5567,18 +6116,29 @@
           <t>MANOEL DE JESUS DE SOUZA MIRANDA ( ZL)</t>
         </is>
       </c>
+      <c r="B41" s="11" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="11" t="inlineStr">
         <is>
-          <t>MARCELO TOMAZ CPF:882.641.062-34</t>
+          <t>MARCELO TOMAZ</t>
+        </is>
+      </c>
+      <c r="B42" s="11" t="inlineStr">
+        <is>
+          <t>88264106234</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="11" t="inlineStr">
         <is>
-          <t>MARLOS  ANDRÉ SILVA RODRIGUES CPF:307.541.782-34</t>
+          <t>MARLOS  ANDRÉ SILVA RODRIGUES</t>
+        </is>
+      </c>
+      <c r="B43" s="11" t="inlineStr">
+        <is>
+          <t>30754178234</t>
         </is>
       </c>
     </row>
@@ -5588,6 +6148,7 @@
           <t>MICILA SUMARIA MEDEIROS PEREIRA</t>
         </is>
       </c>
+      <c r="B44" s="11" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="11" t="inlineStr">
@@ -5595,11 +6156,17 @@
           <t>MITSUO LOPES TAKENO</t>
         </is>
       </c>
+      <c r="B45" s="11" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="11" t="inlineStr">
         <is>
-          <t>PAULO SÉRGIO MENDES DOS SANTOS CPF:021.695.652-80</t>
+          <t>PAULO SÉRGIO MENDES DOS SANTOS</t>
+        </is>
+      </c>
+      <c r="B46" s="11" t="inlineStr">
+        <is>
+          <t>02169565280</t>
         </is>
       </c>
     </row>
@@ -5609,6 +6176,7 @@
           <t>PROF: ALYSSON DE JESUS</t>
         </is>
       </c>
+      <c r="B47" s="11" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="11" t="inlineStr">
@@ -5616,6 +6184,7 @@
           <t>PROF: DAVID RAMOS BRITO, CMZL</t>
         </is>
       </c>
+      <c r="B48" s="11" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="11" t="inlineStr">
@@ -5623,6 +6192,7 @@
           <t>PROF: DAVID RAMOS, CMZL</t>
         </is>
       </c>
+      <c r="B49" s="11" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="11" t="inlineStr">
@@ -5630,6 +6200,7 @@
           <t>PROF: LAURA MICHAELLA</t>
         </is>
       </c>
+      <c r="B50" s="11" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="11" t="inlineStr">
@@ -5637,6 +6208,7 @@
           <t>PROF: MARLOS ANDRE</t>
         </is>
       </c>
+      <c r="B51" s="11" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="11" t="inlineStr">
@@ -5644,11 +6216,17 @@
           <t>PROFESSORA MICILA</t>
         </is>
       </c>
+      <c r="B52" s="11" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="11" t="inlineStr">
         <is>
-          <t>RAGISON DA COSTA DE OLIVEIRA CPF: 014.196.302-61</t>
+          <t>RAGISON DA COSTA DE OLIVEIRA</t>
+        </is>
+      </c>
+      <c r="B53" s="11" t="inlineStr">
+        <is>
+          <t>01419630261</t>
         </is>
       </c>
     </row>
@@ -5658,6 +6236,7 @@
           <t>RAIMUNDO FAGNER</t>
         </is>
       </c>
+      <c r="B54" s="11" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="11" t="inlineStr">
@@ -5665,55 +6244,87 @@
           <t>RAIMUNDO FAGNER COSTA - PROJETO: INOC</t>
         </is>
       </c>
+      <c r="B55" s="11" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="11" t="inlineStr">
         <is>
-          <t>RHAONE GOMES GARCIA CPF: 962.035.102-97</t>
+          <t>RHAONE GOMES GARCIA</t>
+        </is>
+      </c>
+      <c r="B56" s="11" t="inlineStr">
+        <is>
+          <t>96203510297</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="11" t="inlineStr">
         <is>
-          <t>RHAONE GOMES GARCIA CPF: 962.035.102-98</t>
+          <t>RHAONE GOMES GARCIA</t>
+        </is>
+      </c>
+      <c r="B57" s="11" t="inlineStr">
+        <is>
+          <t>96203510298</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="11" t="inlineStr">
         <is>
-          <t>ROCELI PEREIRA LIMA, CPF:337.478.732-00</t>
+          <t>ROCELI PEREIRA LIMA</t>
+        </is>
+      </c>
+      <c r="B58" s="11" t="inlineStr">
+        <is>
+          <t>33747873200</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="11" t="inlineStr">
         <is>
-          <t>VICTORIA SILVA SENEDESE CPF: 009.632.042-70</t>
+          <t>VICTORIA SILVA SENEDESE</t>
+        </is>
+      </c>
+      <c r="B59" s="11" t="inlineStr">
+        <is>
+          <t>00963204270</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="11" t="inlineStr">
         <is>
-          <t>VICTORIA SILVA SENEDESE CPF: 009.632.042-71</t>
+          <t>VICTORIA SILVA SENEDESE</t>
+        </is>
+      </c>
+      <c r="B60" s="11" t="inlineStr">
+        <is>
+          <t>00963204271</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="11" t="inlineStr">
         <is>
-          <t>VITOR BREMGARTNER DA FROTA CPF: 914.180.462-72</t>
+          <t>VITOR BREMGARTNER DA FROTA</t>
+        </is>
+      </c>
+      <c r="B61" s="11" t="inlineStr">
+        <is>
+          <t>91418046272</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="11" t="inlineStr">
         <is>
-          <t>WALTER CLAUDINO DA SILVA JUNIOR SIAPE Nº 3013035</t>
-        </is>
-      </c>
+          <t>WALTER CLAUDINO DA SILVA JUNIOR</t>
+        </is>
+      </c>
+      <c r="B62" s="11" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="11" t="inlineStr">
@@ -5721,6 +6332,7 @@
           <t>WARLEY MATHEUS SANTOS NOGUEIRA</t>
         </is>
       </c>
+      <c r="B63" s="11" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="11" t="inlineStr">
@@ -5728,11 +6340,17 @@
           <t>ZONA LESTE</t>
         </is>
       </c>
+      <c r="B64" s="11" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="11" t="inlineStr">
         <is>
-          <t>ÁLVARO VIANA RIBEIRO CPF:770.465.872-72</t>
+          <t>ÁLVARO VIANA RIBEIRO</t>
+        </is>
+      </c>
+      <c r="B65" s="11" t="inlineStr">
+        <is>
+          <t>77046587272</t>
         </is>
       </c>
     </row>

</xml_diff>